<commit_message>
feat: extend attack range and add ad revival flow
</commit_message>
<xml_diff>
--- a/config/excel/CfgItemDefinitions.xlsx
+++ b/config/excel/CfgItemDefinitions.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgItemDefinitions" sheetId="1" r:id="Raaf96b0467414efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgItemDefinitions" sheetId="1" r:id="R2712bf3f49574c2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="S4" s="20" t="n">
-        <x:v>1.9</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="T4" s="20" t="n">
         <x:v>0</x:v>
@@ -712,7 +712,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="S5" s="20" t="n">
-        <x:v>1.6</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="T5" s="20" t="n">
         <x:v>0.5</x:v>
@@ -901,7 +901,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="S8" s="20" t="n">
-        <x:v>1.35</x:v>
+        <x:v>4.35</x:v>
       </x:c>
       <x:c r="T8" s="20" t="n">
         <x:v>0.2</x:v>
@@ -964,7 +964,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="S9" s="20" t="n">
-        <x:v>2.65</x:v>
+        <x:v>5.65</x:v>
       </x:c>
       <x:c r="T9" s="20" t="n">
         <x:v>0.35</x:v>
@@ -1027,7 +1027,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="S10" s="20" t="n">
-        <x:v>1.65</x:v>
+        <x:v>4.65</x:v>
       </x:c>
       <x:c r="T10" s="20" t="n">
         <x:v>0.25</x:v>

</xml_diff>